<commit_message>
BOM Issues resolved. See #33 for updates.
</commit_message>
<xml_diff>
--- a/Deliverables/Interface_Board/BOM/PCB Way_Interface_Board.xlsx
+++ b/Deliverables/Interface_Board/BOM/PCB Way_Interface_Board.xlsx
@@ -5,7 +5,7 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Github\ChrisitanRaun-AnnanasMotor\Deliverables\Interface_Board\BOM\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\XPENDER\Documents\GitHub\ChristianRaun-EthercatDesign\Deliverables\Interface_Board\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="176" uniqueCount="149">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="176" uniqueCount="148">
   <si>
     <t>Bill of Material (BOM) for Interface_Board</t>
   </si>
@@ -149,26 +149,10 @@
     <t>VKMD1001J101MV</t>
   </si>
   <si>
-    <t>CAP ALUM 10uF 25V SMD</t>
-  </si>
-  <si>
-    <t>RVT1E100M0405</t>
-  </si>
-  <si>
     <t>10uF</t>
   </si>
   <si>
-    <t xml:space="preserve">10V 22uF ±10% CASE-A_3216 Tantalum Capacitors ROHS
-</t>
-  </si>
-  <si>
     <t>C2</t>
-  </si>
-  <si>
-    <t>Cap Case-A</t>
-  </si>
-  <si>
-    <t>CA45A-A-10V-22uF-K</t>
   </si>
   <si>
     <t>22uF</t>
@@ -478,14 +462,26 @@
   </si>
   <si>
     <t>----</t>
+  </si>
+  <si>
+    <t>GRM188R61E106MA73J</t>
+  </si>
+  <si>
+    <t>CAP CER 10UF 25V X5R 0603</t>
+  </si>
+  <si>
+    <t>CAP CER 22UF 25V X5R 0805</t>
+  </si>
+  <si>
+    <t>CC0805MKX5R8BB226</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <numFmts count="1">
-    <numFmt numFmtId="167" formatCode="_-[$$-409]* #,##0.00_ ;_-[$$-409]* \-#,##0.00\ ;_-[$$-409]* &quot;-&quot;??_ ;_-@_ "/>
+    <numFmt numFmtId="164" formatCode="_-[$$-409]* #,##0.00_ ;_-[$$-409]* \-#,##0.00\ ;_-[$$-409]* &quot;-&quot;??_ ;_-@_ "/>
   </numFmts>
   <fonts count="13">
     <font>
@@ -959,7 +955,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="99">
+  <cellXfs count="101">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1181,6 +1177,54 @@
     <xf numFmtId="0" fontId="0" fillId="6" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="4" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="4" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="6" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="11" fillId="6" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="6" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="7" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="7" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1199,53 +1243,11 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="9" fillId="4" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="9" fillId="4" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="9" fillId="6" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="11" fillId="6" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="9" fillId="6" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="9" fillId="7" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="9" fillId="7" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" quotePrefix="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" quotePrefix="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1538,19 +1540,19 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:27" ht="16.5" thickBot="1">
-      <c r="A1" s="80" t="s">
+      <c r="A1" s="96" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="81"/>
-      <c r="C1" s="81"/>
-      <c r="D1" s="81"/>
-      <c r="E1" s="81"/>
-      <c r="F1" s="81"/>
-      <c r="G1" s="81"/>
-      <c r="H1" s="81"/>
-      <c r="I1" s="81"/>
-      <c r="J1" s="81"/>
-      <c r="K1" s="82"/>
+      <c r="B1" s="97"/>
+      <c r="C1" s="97"/>
+      <c r="D1" s="97"/>
+      <c r="E1" s="97"/>
+      <c r="F1" s="97"/>
+      <c r="G1" s="97"/>
+      <c r="H1" s="97"/>
+      <c r="I1" s="97"/>
+      <c r="J1" s="97"/>
+      <c r="K1" s="98"/>
     </row>
     <row r="2" spans="1:27" s="49" customFormat="1" ht="16.5" thickBot="1">
       <c r="A2" s="61" t="s">
@@ -1581,7 +1583,7 @@
         <v>9</v>
       </c>
       <c r="J2" s="51" t="s">
-        <v>144</v>
+        <v>139</v>
       </c>
       <c r="K2" s="51" t="s">
         <v>10</v>
@@ -1607,7 +1609,7 @@
       <c r="A3" s="2">
         <v>1</v>
       </c>
-      <c r="B3" s="77" t="s">
+      <c r="B3" s="93" t="s">
         <v>11</v>
       </c>
       <c r="C3" s="25" t="s">
@@ -1635,13 +1637,13 @@
         <f>I3*5</f>
         <v>20</v>
       </c>
-      <c r="K3" s="83"/>
+      <c r="K3" s="77"/>
     </row>
     <row r="4" spans="1:27" ht="15.75" thickBot="1">
       <c r="A4" s="2">
         <v>2</v>
       </c>
-      <c r="B4" s="78"/>
+      <c r="B4" s="94"/>
       <c r="C4" s="28" t="s">
         <v>17</v>
       </c>
@@ -1667,13 +1669,13 @@
         <f t="shared" ref="J4:J33" si="0">I4*5</f>
         <v>5</v>
       </c>
-      <c r="K4" s="84"/>
+      <c r="K4" s="78"/>
     </row>
     <row r="5" spans="1:27" ht="15.75" thickBot="1">
       <c r="A5" s="2">
         <v>3</v>
       </c>
-      <c r="B5" s="78"/>
+      <c r="B5" s="94"/>
       <c r="C5" s="28" t="s">
         <v>22</v>
       </c>
@@ -1699,13 +1701,13 @@
         <f t="shared" si="0"/>
         <v>40</v>
       </c>
-      <c r="K5" s="84"/>
+      <c r="K5" s="78"/>
     </row>
     <row r="6" spans="1:27" ht="15.75" thickBot="1">
       <c r="A6" s="2">
         <v>4</v>
       </c>
-      <c r="B6" s="78"/>
+      <c r="B6" s="94"/>
       <c r="C6" s="31" t="s">
         <v>26</v>
       </c>
@@ -1731,13 +1733,13 @@
         <f t="shared" si="0"/>
         <v>15</v>
       </c>
-      <c r="K6" s="84"/>
+      <c r="K6" s="78"/>
     </row>
     <row r="7" spans="1:27" ht="15.75" thickBot="1">
       <c r="A7" s="2">
         <v>5</v>
       </c>
-      <c r="B7" s="78"/>
+      <c r="B7" s="94"/>
       <c r="C7" s="31" t="s">
         <v>30</v>
       </c>
@@ -1763,13 +1765,13 @@
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="K7" s="84"/>
+      <c r="K7" s="78"/>
     </row>
     <row r="8" spans="1:27" ht="15.75" thickBot="1">
       <c r="A8" s="2">
         <v>6</v>
       </c>
-      <c r="B8" s="78"/>
+      <c r="B8" s="94"/>
       <c r="C8" s="31" t="s">
         <v>34</v>
       </c>
@@ -1795,13 +1797,13 @@
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="K8" s="85"/>
+      <c r="K8" s="79"/>
     </row>
     <row r="9" spans="1:27" ht="15.75" thickBot="1">
       <c r="A9" s="2">
         <v>7</v>
       </c>
-      <c r="B9" s="78"/>
+      <c r="B9" s="94"/>
       <c r="C9" s="31" t="s">
         <v>39</v>
       </c>
@@ -1827,28 +1829,28 @@
         <f t="shared" si="0"/>
         <v>10</v>
       </c>
-      <c r="K9" s="85"/>
+      <c r="K9" s="79"/>
       <c r="L9" s="22"/>
     </row>
     <row r="10" spans="1:27" ht="15.75" thickBot="1">
       <c r="A10" s="2">
         <v>8</v>
       </c>
-      <c r="B10" s="78"/>
-      <c r="C10" s="31" t="s">
+      <c r="B10" s="94"/>
+      <c r="C10" s="99" t="s">
+        <v>145</v>
+      </c>
+      <c r="D10" s="30" t="s">
+        <v>138</v>
+      </c>
+      <c r="E10" s="32" t="s">
+        <v>14</v>
+      </c>
+      <c r="F10" s="100" t="s">
+        <v>144</v>
+      </c>
+      <c r="G10" s="32" t="s">
         <v>42</v>
-      </c>
-      <c r="D10" s="30" t="s">
-        <v>143</v>
-      </c>
-      <c r="E10" s="32" t="s">
-        <v>36</v>
-      </c>
-      <c r="F10" s="30" t="s">
-        <v>43</v>
-      </c>
-      <c r="G10" s="32" t="s">
-        <v>44</v>
       </c>
       <c r="H10" s="8">
         <v>20</v>
@@ -1860,28 +1862,28 @@
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="K10" s="84"/>
+      <c r="K10" s="78"/>
       <c r="L10" s="22"/>
     </row>
     <row r="11" spans="1:27" ht="15.75" thickBot="1">
       <c r="A11" s="2">
         <v>9</v>
       </c>
-      <c r="B11" s="78"/>
-      <c r="C11" s="31" t="s">
-        <v>45</v>
+      <c r="B11" s="94"/>
+      <c r="C11" s="99" t="s">
+        <v>146</v>
       </c>
       <c r="D11" s="30" t="s">
-        <v>46</v>
-      </c>
-      <c r="E11" s="32" t="s">
-        <v>47</v>
-      </c>
-      <c r="F11" s="30" t="s">
-        <v>48</v>
+        <v>43</v>
+      </c>
+      <c r="E11" s="29" t="s">
+        <v>19</v>
+      </c>
+      <c r="F11" s="100" t="s">
+        <v>147</v>
       </c>
       <c r="G11" s="32" t="s">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="H11" s="8">
         <v>10</v>
@@ -1893,28 +1895,28 @@
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="K11" s="86"/>
+      <c r="K11" s="80"/>
       <c r="L11" s="23"/>
     </row>
     <row r="12" spans="1:27" ht="15.75" thickBot="1">
       <c r="A12" s="2">
         <v>10</v>
       </c>
-      <c r="B12" s="79"/>
+      <c r="B12" s="95"/>
       <c r="C12" s="34" t="s">
-        <v>50</v>
+        <v>45</v>
       </c>
       <c r="D12" s="36" t="s">
-        <v>51</v>
+        <v>46</v>
       </c>
       <c r="E12" s="35" t="s">
-        <v>52</v>
+        <v>47</v>
       </c>
       <c r="F12" s="36" t="s">
-        <v>53</v>
+        <v>48</v>
       </c>
       <c r="G12" s="35" t="s">
-        <v>54</v>
+        <v>49</v>
       </c>
       <c r="H12" s="11">
         <v>50</v>
@@ -1926,30 +1928,30 @@
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="K12" s="87"/>
+      <c r="K12" s="81"/>
       <c r="L12" s="22"/>
     </row>
     <row r="13" spans="1:27" ht="15.75" thickBot="1">
       <c r="A13" s="2">
         <v>11</v>
       </c>
-      <c r="B13" s="77" t="s">
+      <c r="B13" s="93" t="s">
+        <v>50</v>
+      </c>
+      <c r="C13" s="39" t="s">
+        <v>51</v>
+      </c>
+      <c r="D13" s="27" t="s">
+        <v>52</v>
+      </c>
+      <c r="E13" s="40" t="s">
+        <v>53</v>
+      </c>
+      <c r="F13" s="27" t="s">
+        <v>54</v>
+      </c>
+      <c r="G13" s="41" t="s">
         <v>55</v>
-      </c>
-      <c r="C13" s="39" t="s">
-        <v>56</v>
-      </c>
-      <c r="D13" s="27" t="s">
-        <v>57</v>
-      </c>
-      <c r="E13" s="40" t="s">
-        <v>58</v>
-      </c>
-      <c r="F13" s="27" t="s">
-        <v>59</v>
-      </c>
-      <c r="G13" s="41" t="s">
-        <v>60</v>
       </c>
       <c r="H13" s="15">
         <v>7</v>
@@ -1961,28 +1963,28 @@
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="K13" s="83"/>
+      <c r="K13" s="77"/>
       <c r="L13" s="22"/>
     </row>
     <row r="14" spans="1:27" ht="15.75" thickBot="1">
       <c r="A14" s="2">
         <v>12</v>
       </c>
-      <c r="B14" s="79"/>
+      <c r="B14" s="95"/>
       <c r="C14" s="34" t="s">
-        <v>61</v>
+        <v>56</v>
       </c>
       <c r="D14" s="36" t="s">
-        <v>62</v>
+        <v>57</v>
       </c>
       <c r="E14" s="35" t="s">
-        <v>63</v>
+        <v>58</v>
       </c>
       <c r="F14" s="36" t="s">
-        <v>64</v>
+        <v>59</v>
       </c>
       <c r="G14" s="37" t="s">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="H14" s="11">
         <v>20</v>
@@ -1994,7 +1996,7 @@
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="K14" s="88"/>
+      <c r="K14" s="82"/>
       <c r="L14" s="22"/>
     </row>
     <row r="15" spans="1:27" ht="15.75" thickBot="1">
@@ -2002,22 +2004,22 @@
         <v>13</v>
       </c>
       <c r="B15" s="65" t="s">
-        <v>65</v>
+        <v>60</v>
       </c>
       <c r="C15" s="57" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
       <c r="D15" s="54" t="s">
-        <v>67</v>
+        <v>62</v>
       </c>
       <c r="E15" s="54" t="s">
-        <v>68</v>
+        <v>63</v>
       </c>
       <c r="F15" s="54" t="s">
-        <v>69</v>
+        <v>64</v>
       </c>
       <c r="G15" s="52" t="s">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="H15" s="55">
         <v>7</v>
@@ -2029,7 +2031,7 @@
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="K15" s="89"/>
+      <c r="K15" s="83"/>
       <c r="L15" s="22"/>
     </row>
     <row r="16" spans="1:27" ht="15.75" thickBot="1">
@@ -2037,22 +2039,22 @@
         <v>14</v>
       </c>
       <c r="B16" s="64" t="s">
-        <v>70</v>
+        <v>65</v>
       </c>
       <c r="C16" s="60" t="s">
-        <v>71</v>
+        <v>66</v>
       </c>
       <c r="D16" s="58" t="s">
-        <v>72</v>
+        <v>67</v>
       </c>
       <c r="E16" s="58" t="s">
         <v>36</v>
       </c>
       <c r="F16" s="58" t="s">
-        <v>73</v>
+        <v>68</v>
       </c>
       <c r="G16" s="58" t="s">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="H16" s="59">
         <v>7</v>
@@ -2064,30 +2066,30 @@
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="K16" s="90"/>
+      <c r="K16" s="84"/>
       <c r="L16" s="22"/>
     </row>
     <row r="17" spans="1:12" ht="15.75" thickBot="1">
       <c r="A17" s="2">
         <v>15</v>
       </c>
-      <c r="B17" s="77" t="s">
+      <c r="B17" s="93" t="s">
+        <v>69</v>
+      </c>
+      <c r="C17" s="42" t="s">
+        <v>70</v>
+      </c>
+      <c r="D17" s="27" t="s">
+        <v>71</v>
+      </c>
+      <c r="E17" s="27" t="s">
+        <v>72</v>
+      </c>
+      <c r="F17" s="27" t="s">
+        <v>73</v>
+      </c>
+      <c r="G17" s="27" t="s">
         <v>74</v>
-      </c>
-      <c r="C17" s="42" t="s">
-        <v>75</v>
-      </c>
-      <c r="D17" s="27" t="s">
-        <v>76</v>
-      </c>
-      <c r="E17" s="27" t="s">
-        <v>77</v>
-      </c>
-      <c r="F17" s="27" t="s">
-        <v>78</v>
-      </c>
-      <c r="G17" s="27" t="s">
-        <v>79</v>
       </c>
       <c r="H17" s="4">
         <v>100</v>
@@ -2099,28 +2101,28 @@
         <f t="shared" si="0"/>
         <v>10</v>
       </c>
-      <c r="K17" s="91"/>
+      <c r="K17" s="85"/>
       <c r="L17" s="22"/>
     </row>
     <row r="18" spans="1:12" ht="15.75" thickBot="1">
       <c r="A18" s="2">
         <v>16</v>
       </c>
-      <c r="B18" s="78"/>
+      <c r="B18" s="94"/>
       <c r="C18" s="43" t="s">
-        <v>80</v>
+        <v>75</v>
       </c>
       <c r="D18" s="6" t="s">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="E18" s="30" t="s">
+        <v>72</v>
+      </c>
+      <c r="F18" s="30" t="s">
         <v>77</v>
       </c>
-      <c r="F18" s="30" t="s">
-        <v>82</v>
-      </c>
       <c r="G18" s="30" t="s">
-        <v>83</v>
+        <v>78</v>
       </c>
       <c r="H18" s="6">
         <v>100</v>
@@ -2132,28 +2134,28 @@
         <f t="shared" si="0"/>
         <v>10</v>
       </c>
-      <c r="K18" s="92"/>
+      <c r="K18" s="86"/>
       <c r="L18" s="22"/>
     </row>
     <row r="19" spans="1:12" ht="15.75" thickBot="1">
       <c r="A19" s="2">
         <v>17</v>
       </c>
-      <c r="B19" s="78"/>
+      <c r="B19" s="94"/>
       <c r="C19" s="43" t="s">
-        <v>84</v>
+        <v>79</v>
       </c>
       <c r="D19" s="6" t="s">
-        <v>85</v>
+        <v>80</v>
       </c>
       <c r="E19" s="30" t="s">
-        <v>77</v>
+        <v>72</v>
       </c>
       <c r="F19" s="30" t="s">
-        <v>86</v>
+        <v>81</v>
       </c>
       <c r="G19" s="30" t="s">
-        <v>87</v>
+        <v>82</v>
       </c>
       <c r="H19" s="6">
         <v>100</v>
@@ -2165,28 +2167,28 @@
         <f t="shared" si="0"/>
         <v>15</v>
       </c>
-      <c r="K19" s="92"/>
+      <c r="K19" s="86"/>
       <c r="L19" s="22"/>
     </row>
     <row r="20" spans="1:12" ht="15.75" thickBot="1">
       <c r="A20" s="2">
         <v>18</v>
       </c>
-      <c r="B20" s="78"/>
+      <c r="B20" s="94"/>
       <c r="C20" s="43" t="s">
-        <v>88</v>
+        <v>83</v>
       </c>
       <c r="D20" s="30" t="s">
-        <v>89</v>
+        <v>84</v>
       </c>
       <c r="E20" s="30" t="s">
-        <v>90</v>
+        <v>85</v>
       </c>
       <c r="F20" s="30" t="s">
-        <v>91</v>
+        <v>86</v>
       </c>
       <c r="G20" s="30" t="s">
-        <v>92</v>
+        <v>87</v>
       </c>
       <c r="H20" s="6">
         <v>20</v>
@@ -2198,28 +2200,28 @@
         <f t="shared" si="0"/>
         <v>10</v>
       </c>
-      <c r="K20" s="92"/>
+      <c r="K20" s="86"/>
       <c r="L20" s="22"/>
     </row>
     <row r="21" spans="1:12" ht="15.75" thickBot="1">
       <c r="A21" s="2">
         <v>19</v>
       </c>
-      <c r="B21" s="78"/>
+      <c r="B21" s="94"/>
       <c r="C21" s="43" t="s">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="D21" s="30" t="s">
-        <v>94</v>
+        <v>89</v>
       </c>
       <c r="E21" s="30" t="s">
+        <v>85</v>
+      </c>
+      <c r="F21" s="33" t="s">
         <v>90</v>
       </c>
-      <c r="F21" s="33" t="s">
-        <v>95</v>
-      </c>
       <c r="G21" s="30" t="s">
-        <v>96</v>
+        <v>91</v>
       </c>
       <c r="H21" s="6">
         <v>10</v>
@@ -2231,28 +2233,28 @@
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="K21" s="92"/>
+      <c r="K21" s="86"/>
       <c r="L21" s="22"/>
     </row>
     <row r="22" spans="1:12" ht="15.75" thickBot="1">
       <c r="A22" s="2">
         <v>20</v>
       </c>
-      <c r="B22" s="78"/>
+      <c r="B22" s="94"/>
       <c r="C22" s="43" t="s">
-        <v>97</v>
+        <v>92</v>
       </c>
       <c r="D22" s="30" t="s">
-        <v>98</v>
+        <v>93</v>
       </c>
       <c r="E22" s="30" t="s">
         <v>19</v>
       </c>
       <c r="F22" s="30" t="s">
-        <v>99</v>
+        <v>94</v>
       </c>
       <c r="G22" s="30" t="s">
-        <v>100</v>
+        <v>95</v>
       </c>
       <c r="H22" s="6">
         <v>100</v>
@@ -2264,28 +2266,28 @@
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="K22" s="92"/>
+      <c r="K22" s="86"/>
       <c r="L22" s="22"/>
     </row>
     <row r="23" spans="1:12" s="49" customFormat="1" ht="15.75" thickBot="1">
       <c r="A23" s="2">
         <v>21</v>
       </c>
-      <c r="B23" s="79"/>
+      <c r="B23" s="95"/>
       <c r="C23" s="44" t="s">
-        <v>101</v>
+        <v>96</v>
       </c>
       <c r="D23" s="12" t="s">
-        <v>102</v>
+        <v>97</v>
       </c>
       <c r="E23" s="36" t="s">
-        <v>77</v>
+        <v>72</v>
       </c>
       <c r="F23" s="36" t="s">
-        <v>103</v>
+        <v>98</v>
       </c>
       <c r="G23" s="36" t="s">
-        <v>104</v>
+        <v>99</v>
       </c>
       <c r="H23" s="12">
         <v>100</v>
@@ -2297,30 +2299,30 @@
         <f t="shared" si="0"/>
         <v>40</v>
       </c>
-      <c r="K23" s="93"/>
+      <c r="K23" s="87"/>
       <c r="L23" s="63"/>
     </row>
     <row r="24" spans="1:12" ht="15.75" thickBot="1">
       <c r="A24" s="2">
         <v>22</v>
       </c>
-      <c r="B24" s="77" t="s">
-        <v>105</v>
+      <c r="B24" s="93" t="s">
+        <v>100</v>
       </c>
       <c r="C24" s="67" t="s">
-        <v>106</v>
+        <v>101</v>
       </c>
       <c r="D24" s="68" t="s">
-        <v>107</v>
+        <v>102</v>
       </c>
       <c r="E24" s="68" t="s">
-        <v>108</v>
+        <v>103</v>
       </c>
       <c r="F24" s="68" t="s">
-        <v>109</v>
+        <v>104</v>
       </c>
       <c r="G24" s="69" t="s">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="H24" s="70">
         <v>10</v>
@@ -2332,8 +2334,8 @@
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="K24" s="94" t="s">
-        <v>145</v>
+      <c r="K24" s="88" t="s">
+        <v>140</v>
       </c>
       <c r="L24" s="22"/>
     </row>
@@ -2341,21 +2343,21 @@
       <c r="A25" s="2">
         <v>23</v>
       </c>
-      <c r="B25" s="78"/>
+      <c r="B25" s="94"/>
       <c r="C25" s="43" t="s">
-        <v>110</v>
+        <v>105</v>
       </c>
       <c r="D25" s="30" t="s">
-        <v>111</v>
+        <v>106</v>
       </c>
       <c r="E25" s="30" t="s">
-        <v>112</v>
+        <v>107</v>
       </c>
       <c r="F25" s="30" t="s">
-        <v>113</v>
+        <v>108</v>
       </c>
       <c r="G25" s="33" t="s">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="H25" s="10">
         <v>6</v>
@@ -2367,28 +2369,28 @@
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="K25" s="92"/>
+      <c r="K25" s="86"/>
       <c r="L25" s="22"/>
     </row>
     <row r="26" spans="1:12" ht="15.75" thickBot="1">
       <c r="A26" s="2">
         <v>24</v>
       </c>
-      <c r="B26" s="79"/>
+      <c r="B26" s="95"/>
       <c r="C26" s="44" t="s">
-        <v>114</v>
+        <v>109</v>
       </c>
       <c r="D26" s="36" t="s">
-        <v>115</v>
+        <v>110</v>
       </c>
       <c r="E26" s="36" t="s">
-        <v>116</v>
+        <v>111</v>
       </c>
       <c r="F26" s="36" t="s">
-        <v>117</v>
+        <v>112</v>
       </c>
       <c r="G26" s="38" t="s">
-        <v>147</v>
+        <v>142</v>
       </c>
       <c r="H26" s="14">
         <v>6</v>
@@ -2400,30 +2402,30 @@
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="K26" s="88"/>
+      <c r="K26" s="82"/>
       <c r="L26" s="22"/>
     </row>
     <row r="27" spans="1:12" ht="15.75" thickBot="1">
       <c r="A27" s="2">
         <v>25</v>
       </c>
-      <c r="B27" s="77" t="s">
-        <v>118</v>
+      <c r="B27" s="93" t="s">
+        <v>113</v>
       </c>
       <c r="C27" s="67" t="s">
-        <v>119</v>
+        <v>114</v>
       </c>
       <c r="D27" s="68" t="s">
-        <v>120</v>
+        <v>115</v>
       </c>
       <c r="E27" s="68" t="s">
-        <v>121</v>
+        <v>116</v>
       </c>
       <c r="F27" s="68" t="s">
-        <v>121</v>
+        <v>116</v>
       </c>
       <c r="G27" s="68" t="s">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="H27" s="71">
         <v>100</v>
@@ -2435,8 +2437,8 @@
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="K27" s="95" t="s">
-        <v>146</v>
+      <c r="K27" s="89" t="s">
+        <v>141</v>
       </c>
       <c r="L27" s="22"/>
     </row>
@@ -2444,21 +2446,21 @@
       <c r="A28" s="2">
         <v>26</v>
       </c>
-      <c r="B28" s="78"/>
+      <c r="B28" s="94"/>
       <c r="C28" s="72" t="s">
-        <v>122</v>
+        <v>117</v>
       </c>
       <c r="D28" s="73" t="s">
-        <v>123</v>
+        <v>118</v>
       </c>
       <c r="E28" s="73" t="s">
         <v>36</v>
       </c>
       <c r="F28" s="73" t="s">
-        <v>124</v>
+        <v>119</v>
       </c>
       <c r="G28" s="74" t="s">
-        <v>148</v>
+        <v>143</v>
       </c>
       <c r="H28" s="75">
         <v>12</v>
@@ -2470,28 +2472,28 @@
         <f t="shared" si="0"/>
         <v>10</v>
       </c>
-      <c r="K28" s="96"/>
+      <c r="K28" s="90"/>
       <c r="L28" s="22"/>
     </row>
     <row r="29" spans="1:12" ht="15.75" thickBot="1">
       <c r="A29" s="2">
         <v>27</v>
       </c>
-      <c r="B29" s="78"/>
+      <c r="B29" s="94"/>
       <c r="C29" s="72" t="s">
-        <v>125</v>
+        <v>120</v>
       </c>
       <c r="D29" s="73" t="s">
-        <v>126</v>
+        <v>121</v>
       </c>
       <c r="E29" s="73" t="s">
         <v>36</v>
       </c>
       <c r="F29" s="73" t="s">
-        <v>127</v>
+        <v>122</v>
       </c>
       <c r="G29" s="74" t="s">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="H29" s="75">
         <v>10</v>
@@ -2503,28 +2505,28 @@
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="K29" s="96"/>
+      <c r="K29" s="90"/>
       <c r="L29" s="22"/>
     </row>
     <row r="30" spans="1:12" ht="15.75" thickBot="1">
       <c r="A30" s="2">
         <v>28</v>
       </c>
-      <c r="B30" s="78"/>
+      <c r="B30" s="94"/>
       <c r="C30" s="43" t="s">
-        <v>128</v>
+        <v>123</v>
       </c>
       <c r="D30" s="30" t="s">
-        <v>129</v>
+        <v>124</v>
       </c>
       <c r="E30" s="30" t="s">
-        <v>130</v>
+        <v>125</v>
       </c>
       <c r="F30" s="30" t="s">
-        <v>131</v>
+        <v>126</v>
       </c>
       <c r="G30" s="33" t="s">
-        <v>148</v>
+        <v>143</v>
       </c>
       <c r="H30" s="10">
         <v>20</v>
@@ -2536,28 +2538,28 @@
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="K30" s="86"/>
+      <c r="K30" s="80"/>
       <c r="L30" s="22"/>
     </row>
     <row r="31" spans="1:12" ht="15.75" thickBot="1">
       <c r="A31" s="2">
         <v>29</v>
       </c>
-      <c r="B31" s="78"/>
+      <c r="B31" s="94"/>
       <c r="C31" s="43" t="s">
-        <v>132</v>
+        <v>127</v>
       </c>
       <c r="D31" s="30" t="s">
-        <v>133</v>
+        <v>128</v>
       </c>
       <c r="E31" s="30" t="s">
-        <v>134</v>
+        <v>129</v>
       </c>
       <c r="F31" s="30" t="s">
-        <v>135</v>
+        <v>130</v>
       </c>
       <c r="G31" s="33" t="s">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="H31" s="10">
         <v>15</v>
@@ -2569,25 +2571,25 @@
         <f t="shared" si="0"/>
         <v>10</v>
       </c>
-      <c r="K31" s="92"/>
+      <c r="K31" s="86"/>
       <c r="L31" s="22"/>
     </row>
     <row r="32" spans="1:12" ht="15.75" thickBot="1">
       <c r="A32" s="2">
         <v>30</v>
       </c>
-      <c r="B32" s="78"/>
+      <c r="B32" s="94"/>
       <c r="C32" s="45" t="s">
-        <v>136</v>
+        <v>131</v>
       </c>
       <c r="D32" s="16" t="s">
-        <v>137</v>
+        <v>132</v>
       </c>
       <c r="E32" s="46" t="s">
-        <v>138</v>
+        <v>133</v>
       </c>
       <c r="F32" s="16" t="s">
-        <v>138</v>
+        <v>133</v>
       </c>
       <c r="G32" s="16"/>
       <c r="H32" s="16"/>
@@ -2598,8 +2600,8 @@
         <f t="shared" si="0"/>
         <v>25</v>
       </c>
-      <c r="K32" s="97" t="s">
-        <v>139</v>
+      <c r="K32" s="91" t="s">
+        <v>134</v>
       </c>
       <c r="L32" s="22"/>
     </row>
@@ -2607,18 +2609,18 @@
       <c r="A33" s="53">
         <v>31</v>
       </c>
-      <c r="B33" s="79"/>
+      <c r="B33" s="95"/>
       <c r="C33" s="47" t="s">
-        <v>140</v>
+        <v>135</v>
       </c>
       <c r="D33" s="17" t="s">
-        <v>141</v>
+        <v>136</v>
       </c>
       <c r="E33" s="48" t="s">
-        <v>142</v>
+        <v>137</v>
       </c>
       <c r="F33" s="17" t="s">
-        <v>142</v>
+        <v>137</v>
       </c>
       <c r="G33" s="17"/>
       <c r="H33" s="17"/>
@@ -2629,8 +2631,8 @@
         <f t="shared" si="0"/>
         <v>25</v>
       </c>
-      <c r="K33" s="98" t="s">
-        <v>139</v>
+      <c r="K33" s="92" t="s">
+        <v>134</v>
       </c>
       <c r="L33" s="22"/>
     </row>

</xml_diff>